<commit_message>
Rename project to MethodMesh
</commit_message>
<xml_diff>
--- a/docs/examples/example_odk_nfc_credential_provisioning.xlsx
+++ b/docs/examples/example_odk_nfc_credential_provisioning.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="survey" sheetId="1" r:id="R82a102b333884e7e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="choices" sheetId="2" r:id="R1ee950cd9f894bbe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settings" sheetId="3" r:id="R5c396551c38a4395"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="survey" sheetId="1" r:id="Rb6f05dd819a44d11"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="choices" sheetId="2" r:id="R5808f743793f4912"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settings" sheetId="3" r:id="R521cd053816b4bbb"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -349,7 +349,7 @@
         <x:v>Provision a portable NFC credential</x:v>
       </x:c>
       <x:c r="D4" s="3" t="str">
-        <x:v>ResearchOS scans the card, asks for a 4- or 6-digit PIN, then asks for the same card again to write and verify the encrypted credential.</x:v>
+        <x:v>MethodMesh scans the card, asks for a 4- or 6-digit PIN, then asks for the same card again to write and verify the encrypted credential.</x:v>
       </x:c>
       <x:c r="E4" s="3" t="str"/>
       <x:c r="F4" s="3" t="str"/>
@@ -389,7 +389,7 @@
         <x:v>PIN length</x:v>
       </x:c>
       <x:c r="D6" s="3" t="str">
-        <x:v>The person creates and enters the PIN inside ResearchOS; the PIN is never returned to this form.</x:v>
+        <x:v>The person creates and enters the PIN inside MethodMesh; the PIN is never returned to this form.</x:v>
       </x:c>
       <x:c r="E6" s="3" t="str"/>
       <x:c r="F6" s="3" t="str"/>
@@ -437,7 +437,7 @@
         <x:v>field-list</x:v>
       </x:c>
       <x:c r="F8" s="3" t="str">
-        <x:v>com.example.researchos.EXECUTE_METHOD(method_id='nfc_credential_provisioning',input_credential_subject_id=${credential_subject_id_input},input_pin_length=${pin_length_input},input_overwrite_policy=${overwrite_policy_input},return_mode='flat')</x:v>
+        <x:v>com.example.methodmesh.EXECUTE_METHOD(method_id='nfc_credential_provisioning',input_credential_subject_id=${credential_subject_id_input},input_pin_length=${pin_length_input},input_overwrite_policy=${overwrite_policy_input},return_mode='flat')</x:v>
       </x:c>
       <x:c r="G8" s="3" t="str"/>
       <x:c r="H8" s="3" t="str"/>
@@ -448,10 +448,10 @@
         <x:v>text</x:v>
       </x:c>
       <x:c r="B9" s="3" t="str">
-        <x:v>researchos_execution_id</x:v>
+        <x:v>methodmesh_execution_id</x:v>
       </x:c>
       <x:c r="C9" s="3" t="str">
-        <x:v>ResearchOS execution ID</x:v>
+        <x:v>MethodMesh execution ID</x:v>
       </x:c>
       <x:c r="D9" s="3" t="str"/>
       <x:c r="E9" s="3" t="str"/>
@@ -465,10 +465,10 @@
         <x:v>text</x:v>
       </x:c>
       <x:c r="B10" s="3" t="str">
-        <x:v>researchos_status</x:v>
+        <x:v>methodmesh_status</x:v>
       </x:c>
       <x:c r="C10" s="3" t="str">
-        <x:v>ResearchOS status</x:v>
+        <x:v>MethodMesh status</x:v>
       </x:c>
       <x:c r="D10" s="3" t="str"/>
       <x:c r="E10" s="3" t="str"/>

</xml_diff>